<commit_message>
fix(formula): ignore blanks in average ranges
</commit_message>
<xml_diff>
--- a/packages/headless/fixtures/xlsx-corpus/issue-8-production-regressions.xlsx
+++ b/packages/headless/fixtures/xlsx-corpus/issue-8-production-regressions.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="Activity" sheetId="2" r:id="rId2"/>
     <sheet name="Bank" sheetId="3" r:id="rId3"/>
+    <sheet name="AverageInputs" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -518,6 +519,15 @@
         <v>2026-04-01</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Average ignores blanks</v>
+      </c>
+      <c r="B13">
+        <f>ROUND(AVERAGE(AverageInputs!$A$2:$A$20),2)</f>
+        <v>18.91</v>
+      </c>
+    </row>
     <row r="14">
       <c r="A14" t="str">
         <v>Bank lookup</v>
@@ -617,4 +627,55 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D31"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A20"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Value</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>18.75</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>20.25</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>19.04</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Department</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A20"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>